<commit_message>
Update generation outputs, docs, gates, and presentation
</commit_message>
<xml_diff>
--- a/outputs/generated/nitro_bioisostere_campaign/mol2mol_mmp/plain/mol2mol_mmp_plain_generated_optimal.xlsx
+++ b/outputs/generated/nitro_bioisostere_campaign/mol2mol_mmp/plain/mol2mol_mmp_plain_generated_optimal.xlsx
@@ -652,23 +652,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:BF8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" customWidth="1"/>
     <col min="3" max="4" width="14.7109375" customWidth="1"/>
     <col min="5" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" customWidth="1"/>
-    <col min="9" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" customWidth="1"/>
-    <col min="12" max="12" width="32.7109375" customWidth="1"/>
-    <col min="13" max="13" width="28.7109375" customWidth="1"/>
-    <col min="14" max="14" width="37.7109375" customWidth="1"/>
-    <col min="15" max="15" width="38.7109375" customWidth="1"/>
-    <col min="16" max="16" width="30.7109375" customWidth="1"/>
-    <col min="17" max="17" width="16.7109375" customWidth="1"/>
+    <col min="7" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="31.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" customWidth="1"/>
+    <col min="14" max="14" width="28.7109375" customWidth="1"/>
+    <col min="15" max="15" width="27.7109375" customWidth="1"/>
+    <col min="16" max="16" width="26.7109375" customWidth="1"/>
+    <col min="17" max="17" width="25.7109375" customWidth="1"/>
+    <col min="18" max="19" width="22.7109375" customWidth="1"/>
+    <col min="20" max="21" width="20.7109375" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" customWidth="1"/>
+    <col min="24" max="24" width="16.7109375" customWidth="1"/>
+    <col min="25" max="25" width="32.7109375" customWidth="1"/>
+    <col min="26" max="26" width="28.7109375" customWidth="1"/>
+    <col min="27" max="27" width="37.7109375" customWidth="1"/>
+    <col min="28" max="28" width="38.7109375" customWidth="1"/>
+    <col min="29" max="29" width="30.7109375" customWidth="1"/>
+    <col min="30" max="31" width="13.7109375" customWidth="1"/>
+    <col min="32" max="35" width="12.7109375" customWidth="1"/>
+    <col min="36" max="36" width="21.7109375" customWidth="1"/>
+    <col min="37" max="37" width="12.7109375" customWidth="1"/>
+    <col min="38" max="38" width="14.7109375" customWidth="1"/>
+    <col min="39" max="39" width="15.7109375" customWidth="1"/>
+    <col min="40" max="42" width="14.7109375" customWidth="1"/>
+    <col min="43" max="43" width="12.7109375" customWidth="1"/>
+    <col min="44" max="44" width="20.7109375" customWidth="1"/>
+    <col min="45" max="45" width="13.7109375" customWidth="1"/>
+    <col min="46" max="46" width="17.7109375" customWidth="1"/>
+    <col min="47" max="48" width="12.7109375" customWidth="1"/>
+    <col min="49" max="49" width="15.7109375" customWidth="1"/>
+    <col min="50" max="50" width="18.7109375" customWidth="1"/>
+    <col min="51" max="54" width="12.7109375" customWidth="1"/>
+    <col min="55" max="55" width="18.7109375" customWidth="1"/>
+    <col min="56" max="56" width="23.7109375" customWidth="1"/>
+    <col min="57" max="57" width="25.7109375" customWidth="1"/>
+    <col min="58" max="58" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -704,55 +733,260 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>qsar_model_count</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>qsar_models_used</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>pred_logIC50_uM</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pred_ic50_uM</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pred_pIC50</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>pred_logIC50_uM_ensemble_mean</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>pred_logIC50_uM_ensemble_std</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>pred_ic50_uM_ensemble_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>pred_ic50_uM_ensemble_std</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>pred_pIC50_ensemble_mean</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>pred_pIC50_ensemble_std</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>pred_ic50_uM_lower95</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>pred_ic50_uM_upper95</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>pred_pIC50_lower95</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>pred_pIC50_upper95</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>pred_pIC50_uncertainty</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>pred_cLogP</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>pred_logS_ESOL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>pred_Solubility_ESOL_mol_per_L</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>pred_Solubility_ESOL_class</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>pred_MetStab_Clearance_Microsome_AZ</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>pred_MetStab_Clearance_Hepatocyte_AZ</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>pred_MetStab_Half_Life_Obach</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>PAINS_alert</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>BRENK_alert</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>NIH_alert</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>AMES</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>ClinTox</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>DILI</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Carcinogens_Lagunin</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>hERG</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>CYP1A2_Veith</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>CYP2C19_Veith</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>CYP2C9_Veith</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>CYP2D6_Veith</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>CYP3A4_Veith</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>HIA_Hou</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Bioavailability_Ma</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>PAMPA_NCATS</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Pgp_Broccatelli</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Caco2_Wang</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>PPBR_AZ</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>VDss_Lombardo</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>molecular_weight</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>logP</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>QED</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Lipinski</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>sa_score</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>sa_accessibility</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>liability_alert_count</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>passes_qsar_uncertainty</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>passes_optimal</t>
         </is>
@@ -779,38 +1013,163 @@
         <v>12.53</v>
       </c>
       <c r="G2" s="3">
-        <v>0.6736750368070121</v>
-      </c>
-      <c r="H2" s="3">
-        <v>4.717099496597866</v>
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I2" s="3">
-        <v>5.326324963192988</v>
+        <v>0.6736750385683135</v>
       </c>
       <c r="J2" s="3">
+        <v>4.717099515728281</v>
+      </c>
+      <c r="K2" s="3">
+        <v>5.326324961431687</v>
+      </c>
+      <c r="L2" s="3">
+        <v>1.196034223649022</v>
+      </c>
+      <c r="M2" s="3">
+        <v>0.5831712914652263</v>
+      </c>
+      <c r="N2" s="3">
+        <v>47.50124066547174</v>
+      </c>
+      <c r="O2" s="3">
+        <v>76.37014685823269</v>
+      </c>
+      <c r="P2" s="3">
+        <v>4.803965776350978</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>0.5831712914652263</v>
+      </c>
+      <c r="R2" s="3">
+        <v>1.129844022714398</v>
+      </c>
+      <c r="S2" s="3">
+        <v>218.2980995786917</v>
+      </c>
+      <c r="T2" s="3">
+        <v>3.660950045079134</v>
+      </c>
+      <c r="U2" s="3">
+        <v>5.946981507622821</v>
+      </c>
+      <c r="V2" s="3">
+        <v>0.5831712914652263</v>
+      </c>
+      <c r="W2" s="3">
         <v>3.179500000000001</v>
       </c>
-      <c r="K2" s="3">
+      <c r="X2" s="3">
         <v>-4.697726188509208</v>
       </c>
-      <c r="L2" s="3">
+      <c r="Y2" s="3">
         <v>2.005736193847606E-05</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N2" s="3">
+      <c r="AA2" s="3">
         <v>44.49736785888672</v>
       </c>
-      <c r="O2" s="3">
+      <c r="AB2" s="3">
         <v>36.57278060913086</v>
       </c>
-      <c r="P2" s="3">
+      <c r="AC2" s="3">
         <v>42.2242431640625</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="AD2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="3">
+        <v>0.1213474124670029</v>
+      </c>
+      <c r="AH2" s="3">
+        <v>0.3793679773807526</v>
+      </c>
+      <c r="AI2" s="3">
+        <v>0.6308319568634033</v>
+      </c>
+      <c r="AJ2" s="3">
+        <v>0.06799260526895523</v>
+      </c>
+      <c r="AK2" s="3">
+        <v>0.8862754702568054</v>
+      </c>
+      <c r="AL2" s="3">
+        <v>0.1875756233930588</v>
+      </c>
+      <c r="AM2" s="3">
+        <v>0.4857034087181091</v>
+      </c>
+      <c r="AN2" s="3">
+        <v>0.5998517274856567</v>
+      </c>
+      <c r="AO2" s="3">
+        <v>0.1621912717819214</v>
+      </c>
+      <c r="AP2" s="3">
+        <v>0.9689401388168335</v>
+      </c>
+      <c r="AQ2" s="3">
+        <v>0.9997833967208862</v>
+      </c>
+      <c r="AR2" s="3">
+        <v>0.7327489852905273</v>
+      </c>
+      <c r="AS2" s="3">
+        <v>0.9529389142990112</v>
+      </c>
+      <c r="AT2" s="3">
+        <v>0.8042116165161133</v>
+      </c>
+      <c r="AU2" s="3">
+        <v>-4.799037456512451</v>
+      </c>
+      <c r="AV2" s="3">
+        <v>94.31733703613281</v>
+      </c>
+      <c r="AW2" s="3">
+        <v>12.37920379638672</v>
+      </c>
+      <c r="AX2" s="3">
+        <v>382.5520000000002</v>
+      </c>
+      <c r="AY2" s="3">
+        <v>3.179500000000001</v>
+      </c>
+      <c r="AZ2" s="3">
+        <v>0.6062696116808681</v>
+      </c>
+      <c r="BA2" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB2" s="3">
+        <v>3.517572745759535</v>
+      </c>
+      <c r="BC2" s="3">
+        <v>0.7202696949156071</v>
+      </c>
+      <c r="BD2" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE2" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF2" s="3">
         <v>1</v>
       </c>
     </row>
@@ -835,38 +1194,163 @@
         <v>9.66</v>
       </c>
       <c r="G3" s="3">
-        <v>0.6922399224099494</v>
-      </c>
-      <c r="H3" s="3">
-        <v>4.923114339678773</v>
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I3" s="3">
-        <v>5.307760077590051</v>
+        <v>0.6922399241634253</v>
       </c>
       <c r="J3" s="3">
+        <v>4.923114359555983</v>
+      </c>
+      <c r="K3" s="3">
+        <v>5.307760075836574</v>
+      </c>
+      <c r="L3" s="3">
+        <v>1.245024441083629</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0.5927358158413236</v>
+      </c>
+      <c r="N3" s="3">
+        <v>49.97127390291917</v>
+      </c>
+      <c r="O3" s="3">
+        <v>75.51939823741807</v>
+      </c>
+      <c r="P3" s="3">
+        <v>4.754975558916371</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>0.5927358158413236</v>
+      </c>
+      <c r="R3" s="3">
+        <v>1.211329355336148</v>
+      </c>
+      <c r="S3" s="3">
+        <v>255.1447521483189</v>
+      </c>
+      <c r="T3" s="3">
+        <v>3.593213359867377</v>
+      </c>
+      <c r="U3" s="3">
+        <v>5.916737757965365</v>
+      </c>
+      <c r="V3" s="3">
+        <v>0.5927358158413236</v>
+      </c>
+      <c r="W3" s="3">
         <v>3.461900000000001</v>
       </c>
-      <c r="K3" s="3">
+      <c r="X3" s="3">
         <v>-5.488866073692056</v>
       </c>
-      <c r="L3" s="3">
+      <c r="Y3" s="3">
         <v>3.244396515601069E-06</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="Z3" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N3" s="3">
+      <c r="AA3" s="3">
         <v>56.6396598815918</v>
       </c>
-      <c r="O3" s="3">
+      <c r="AB3" s="3">
         <v>48.72274017333984</v>
       </c>
-      <c r="P3" s="3">
-        <v>43.81204223632812</v>
-      </c>
-      <c r="Q3" s="3">
+      <c r="AC3" s="3">
+        <v>43.81204986572266</v>
+      </c>
+      <c r="AD3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF3" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="3">
+        <v>0.2192052155733109</v>
+      </c>
+      <c r="AH3" s="3">
+        <v>0.4016119837760925</v>
+      </c>
+      <c r="AI3" s="3">
+        <v>0.897729218006134</v>
+      </c>
+      <c r="AJ3" s="3">
+        <v>0.07054200768470764</v>
+      </c>
+      <c r="AK3" s="3">
+        <v>0.9418826103210449</v>
+      </c>
+      <c r="AL3" s="3">
+        <v>0.4947546124458313</v>
+      </c>
+      <c r="AM3" s="3">
+        <v>0.8435236811637878</v>
+      </c>
+      <c r="AN3" s="3">
+        <v>0.9229615330696106</v>
+      </c>
+      <c r="AO3" s="3">
+        <v>0.2877492904663086</v>
+      </c>
+      <c r="AP3" s="3">
+        <v>0.9939088821411133</v>
+      </c>
+      <c r="AQ3" s="3">
+        <v>0.9999846220016479</v>
+      </c>
+      <c r="AR3" s="3">
+        <v>0.726409375667572</v>
+      </c>
+      <c r="AS3" s="3">
+        <v>0.9672144651412964</v>
+      </c>
+      <c r="AT3" s="3">
+        <v>0.9312014579772949</v>
+      </c>
+      <c r="AU3" s="3">
+        <v>-4.826889991760254</v>
+      </c>
+      <c r="AV3" s="3">
+        <v>102.379753112793</v>
+      </c>
+      <c r="AW3" s="3">
+        <v>6.813174247741699</v>
+      </c>
+      <c r="AX3" s="3">
+        <v>461.5660000000003</v>
+      </c>
+      <c r="AY3" s="3">
+        <v>3.461900000000001</v>
+      </c>
+      <c r="AZ3" s="3">
+        <v>0.5200375068799599</v>
+      </c>
+      <c r="BA3" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB3" s="3">
+        <v>3.713919171191669</v>
+      </c>
+      <c r="BC3" s="3">
+        <v>0.6984534254231478</v>
+      </c>
+      <c r="BD3" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE3" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="3">
         <v>1</v>
       </c>
     </row>
@@ -891,45 +1375,170 @@
         <v>11.87</v>
       </c>
       <c r="G4" s="3">
-        <v>0.6976196057554537</v>
-      </c>
-      <c r="H4" s="3">
-        <v>4.984477107800574</v>
+        <v>5</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I4" s="3">
-        <v>5.302380394244547</v>
+        <v>0.6976196075069575</v>
       </c>
       <c r="J4" s="3">
+        <v>4.984477127902903</v>
+      </c>
+      <c r="K4" s="3">
+        <v>5.302380392493043</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0.8836030068125652</v>
+      </c>
+      <c r="M4" s="3">
+        <v>0.1803645338738968</v>
+      </c>
+      <c r="N4" s="3">
+        <v>8.32240433842561</v>
+      </c>
+      <c r="O4" s="3">
+        <v>3.344459505055267</v>
+      </c>
+      <c r="P4" s="3">
+        <v>5.116396993187434</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>0.1803645338738968</v>
+      </c>
+      <c r="R4" s="3">
+        <v>3.38913228359138</v>
+      </c>
+      <c r="S4" s="3">
+        <v>17.26304860063566</v>
+      </c>
+      <c r="T4" s="3">
+        <v>4.762882506794597</v>
+      </c>
+      <c r="U4" s="3">
+        <v>5.469911479580272</v>
+      </c>
+      <c r="V4" s="3">
+        <v>0.1803645338738968</v>
+      </c>
+      <c r="W4" s="3">
         <v>3.478700000000003</v>
       </c>
-      <c r="K4" s="3">
+      <c r="X4" s="3">
         <v>-5.002432848934182</v>
       </c>
-      <c r="L4" s="3">
+      <c r="Y4" s="3">
         <v>9.944138193685663E-06</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="Z4" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N4" s="3">
+      <c r="AA4" s="3">
         <v>53.13448333740234</v>
       </c>
-      <c r="O4" s="3">
+      <c r="AB4" s="3">
         <v>56.53021240234375</v>
       </c>
-      <c r="P4" s="3">
+      <c r="AC4" s="3">
         <v>44.11494064331055</v>
       </c>
-      <c r="Q4" s="3">
+      <c r="AD4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF4" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="3">
+        <v>0.2469469308853149</v>
+      </c>
+      <c r="AH4" s="3">
+        <v>0.2810777425765991</v>
+      </c>
+      <c r="AI4" s="3">
+        <v>0.6463785171508789</v>
+      </c>
+      <c r="AJ4" s="3">
+        <v>0.05409278720617294</v>
+      </c>
+      <c r="AK4" s="3">
+        <v>0.8009153604507446</v>
+      </c>
+      <c r="AL4" s="3">
+        <v>0.206072524189949</v>
+      </c>
+      <c r="AM4" s="3">
+        <v>0.5045340061187744</v>
+      </c>
+      <c r="AN4" s="3">
+        <v>0.5027914643287659</v>
+      </c>
+      <c r="AO4" s="3">
+        <v>0.09001477062702179</v>
+      </c>
+      <c r="AP4" s="3">
+        <v>0.9486678838729858</v>
+      </c>
+      <c r="AQ4" s="3">
+        <v>0.9999431371688843</v>
+      </c>
+      <c r="AR4" s="3">
+        <v>0.7472778558731079</v>
+      </c>
+      <c r="AS4" s="3">
+        <v>0.9748571515083313</v>
+      </c>
+      <c r="AT4" s="3">
+        <v>0.7642152309417725</v>
+      </c>
+      <c r="AU4" s="3">
+        <v>-4.632003784179688</v>
+      </c>
+      <c r="AV4" s="3">
+        <v>97.15895843505859</v>
+      </c>
+      <c r="AW4" s="3">
+        <v>10.61889266967773</v>
+      </c>
+      <c r="AX4" s="3">
+        <v>395.5470000000003</v>
+      </c>
+      <c r="AY4" s="3">
+        <v>3.478700000000003</v>
+      </c>
+      <c r="AZ4" s="3">
+        <v>0.5464877990227248</v>
+      </c>
+      <c r="BA4" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB4" s="3">
+        <v>3.868812272151152</v>
+      </c>
+      <c r="BC4" s="3">
+        <v>0.6812430808720943</v>
+      </c>
+      <c r="BD4" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE4" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="5" ht="92" customHeight="1">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4cc[nH]n4)C3)C2)c1</t>
+          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4cnn(C)c4)C3)C2)c1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -941,51 +1550,176 @@
         <v>1</v>
       </c>
       <c r="E5" s="3">
-        <v>0.6228070175438597</v>
+        <v>0.6403508771929824</v>
       </c>
       <c r="F5" s="3">
-        <v>12.75</v>
+        <v>10.99</v>
       </c>
       <c r="G5" s="3">
-        <v>0.6976196057554537</v>
-      </c>
-      <c r="H5" s="3">
-        <v>4.984477107800574</v>
+        <v>5</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I5" s="3">
-        <v>5.302380394244547</v>
+        <v>0.6976196075069575</v>
       </c>
       <c r="J5" s="3">
-        <v>3.479100000000002</v>
+        <v>4.984477127902903</v>
       </c>
       <c r="K5" s="3">
-        <v>-5.04957989485515</v>
+        <v>5.302380392493043</v>
       </c>
       <c r="L5" s="3">
-        <v>8.921134870987701E-06</v>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
+        <v>1.087896721431184</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0.2832139466588319</v>
+      </c>
+      <c r="N5" s="3">
+        <v>14.99202021366446</v>
+      </c>
+      <c r="O5" s="3">
+        <v>9.017290093260467</v>
+      </c>
+      <c r="P5" s="3">
+        <v>4.912103278568816</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>0.2832139466588319</v>
+      </c>
+      <c r="R5" s="3">
+        <v>3.410337699636223</v>
+      </c>
+      <c r="S5" s="3">
+        <v>43.95376246978022</v>
+      </c>
+      <c r="T5" s="3">
+        <v>4.357003943117506</v>
+      </c>
+      <c r="U5" s="3">
+        <v>5.467202614020127</v>
+      </c>
+      <c r="V5" s="3">
+        <v>0.2832139466588319</v>
+      </c>
+      <c r="W5" s="3">
+        <v>3.489500000000002</v>
+      </c>
+      <c r="X5" s="3">
+        <v>-5.14467691804052</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>7.166763644850975E-06</v>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N5" s="3">
-        <v>62.83623123168945</v>
-      </c>
-      <c r="O5" s="3">
-        <v>60.1665153503418</v>
-      </c>
-      <c r="P5" s="3">
-        <v>48.18215179443359</v>
-      </c>
-      <c r="Q5" s="3">
+      <c r="AA5" s="3">
+        <v>54.14443206787109</v>
+      </c>
+      <c r="AB5" s="3">
+        <v>48.61449813842773</v>
+      </c>
+      <c r="AC5" s="3">
+        <v>42.2707405090332</v>
+      </c>
+      <c r="AD5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="3">
+        <v>0.1222689300775528</v>
+      </c>
+      <c r="AH5" s="3">
+        <v>0.2155998200178146</v>
+      </c>
+      <c r="AI5" s="3">
+        <v>0.8456916809082031</v>
+      </c>
+      <c r="AJ5" s="3">
+        <v>0.06358656287193298</v>
+      </c>
+      <c r="AK5" s="3">
+        <v>0.760409951210022</v>
+      </c>
+      <c r="AL5" s="3">
+        <v>0.2809678912162781</v>
+      </c>
+      <c r="AM5" s="3">
+        <v>0.5562871098518372</v>
+      </c>
+      <c r="AN5" s="3">
+        <v>0.7078112363815308</v>
+      </c>
+      <c r="AO5" s="3">
+        <v>0.05011356994509697</v>
+      </c>
+      <c r="AP5" s="3">
+        <v>0.9613454937934875</v>
+      </c>
+      <c r="AQ5" s="3">
+        <v>0.9999285936355591</v>
+      </c>
+      <c r="AR5" s="3">
+        <v>0.8209438323974609</v>
+      </c>
+      <c r="AS5" s="3">
+        <v>0.968595027923584</v>
+      </c>
+      <c r="AT5" s="3">
+        <v>0.7425563931465149</v>
+      </c>
+      <c r="AU5" s="3">
+        <v>-4.84219217300415</v>
+      </c>
+      <c r="AV5" s="3">
+        <v>98.20294189453125</v>
+      </c>
+      <c r="AW5" s="3">
+        <v>9.877103805541992</v>
+      </c>
+      <c r="AX5" s="3">
+        <v>405.5460000000002</v>
+      </c>
+      <c r="AY5" s="3">
+        <v>3.489500000000002</v>
+      </c>
+      <c r="AZ5" s="3">
+        <v>0.5453323613042372</v>
+      </c>
+      <c r="BA5" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB5" s="3">
+        <v>3.415974062512648</v>
+      </c>
+      <c r="BC5" s="3">
+        <v>0.7315584374985946</v>
+      </c>
+      <c r="BD5" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE5" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF5" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="6" ht="92" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4ccc(S(N)(=O)=O)cc4)C3)C2)c1</t>
+          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4ccnn4C)C3)C2)c1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -997,51 +1731,176 @@
         <v>1</v>
       </c>
       <c r="E6" s="3">
-        <v>0.6416666666666667</v>
+        <v>0.6120689655172413</v>
       </c>
       <c r="F6" s="3">
-        <v>9.01</v>
+        <v>10.3</v>
       </c>
       <c r="G6" s="3">
-        <v>0.6976196057554538</v>
-      </c>
-      <c r="H6" s="3">
-        <v>4.984477107800576</v>
+        <v>5</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I6" s="3">
-        <v>5.302380394244546</v>
+        <v>0.6976196075069575</v>
       </c>
       <c r="J6" s="3">
-        <v>3.403400000000001</v>
+        <v>4.984477127902903</v>
       </c>
       <c r="K6" s="3">
-        <v>-5.568140156782245</v>
+        <v>5.302380392493043</v>
       </c>
       <c r="L6" s="3">
-        <v>2.703085875570429E-06</v>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
+        <v>1.077329349319045</v>
+      </c>
+      <c r="M6" s="3">
+        <v>0.3004071563362712</v>
+      </c>
+      <c r="N6" s="3">
+        <v>15.02157122362034</v>
+      </c>
+      <c r="O6" s="3">
+        <v>9.557065069708871</v>
+      </c>
+      <c r="P6" s="3">
+        <v>4.922670650680955</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>0.3004071563362712</v>
+      </c>
+      <c r="R6" s="3">
+        <v>3.079862464391477</v>
+      </c>
+      <c r="S6" s="3">
+        <v>46.35828656292931</v>
+      </c>
+      <c r="T6" s="3">
+        <v>4.333872624261863</v>
+      </c>
+      <c r="U6" s="3">
+        <v>5.511468677100047</v>
+      </c>
+      <c r="V6" s="3">
+        <v>0.3004071563362712</v>
+      </c>
+      <c r="W6" s="3">
+        <v>3.489500000000002</v>
+      </c>
+      <c r="X6" s="3">
+        <v>-5.14467691804052</v>
+      </c>
+      <c r="Y6" s="3">
+        <v>7.166763644850975E-06</v>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N6" s="3">
-        <v>43.70171356201172</v>
-      </c>
-      <c r="O6" s="3">
-        <v>27.25896072387695</v>
-      </c>
-      <c r="P6" s="3">
-        <v>48.61517333984375</v>
-      </c>
-      <c r="Q6" s="3">
+      <c r="AA6" s="3">
+        <v>62.84810638427734</v>
+      </c>
+      <c r="AB6" s="3">
+        <v>55.03955078125</v>
+      </c>
+      <c r="AC6" s="3">
+        <v>48.48752593994141</v>
+      </c>
+      <c r="AD6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE6" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="3">
+        <v>0.1596864759922028</v>
+      </c>
+      <c r="AH6" s="3">
+        <v>0.2792690992355347</v>
+      </c>
+      <c r="AI6" s="3">
+        <v>0.8238638043403625</v>
+      </c>
+      <c r="AJ6" s="3">
+        <v>0.0565599612891674</v>
+      </c>
+      <c r="AK6" s="3">
+        <v>0.8657090067863464</v>
+      </c>
+      <c r="AL6" s="3">
+        <v>0.4318308234214783</v>
+      </c>
+      <c r="AM6" s="3">
+        <v>0.7112659215927124</v>
+      </c>
+      <c r="AN6" s="3">
+        <v>0.8083459734916687</v>
+      </c>
+      <c r="AO6" s="3">
+        <v>0.1134422272443771</v>
+      </c>
+      <c r="AP6" s="3">
+        <v>0.987573504447937</v>
+      </c>
+      <c r="AQ6" s="3">
+        <v>0.9999877214431763</v>
+      </c>
+      <c r="AR6" s="3">
+        <v>0.7667804956436157</v>
+      </c>
+      <c r="AS6" s="3">
+        <v>0.9786069989204407</v>
+      </c>
+      <c r="AT6" s="3">
+        <v>0.8238350749015808</v>
+      </c>
+      <c r="AU6" s="3">
+        <v>-4.787118434906006</v>
+      </c>
+      <c r="AV6" s="3">
+        <v>99.26639556884766</v>
+      </c>
+      <c r="AW6" s="3">
+        <v>10.56526756286621</v>
+      </c>
+      <c r="AX6" s="3">
+        <v>405.5460000000002</v>
+      </c>
+      <c r="AY6" s="3">
+        <v>3.489500000000002</v>
+      </c>
+      <c r="AZ6" s="3">
+        <v>0.5453323613042372</v>
+      </c>
+      <c r="BA6" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB6" s="3">
+        <v>3.45885205893483</v>
+      </c>
+      <c r="BC6" s="3">
+        <v>0.7267942156739078</v>
+      </c>
+      <c r="BD6" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE6" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF6" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4ccnn4C)C3)C2)c1</t>
+          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4ccc(S(N)(=O)=O)cc4)C3)C2)c1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1053,51 +1912,176 @@
         <v>1</v>
       </c>
       <c r="E7" s="3">
-        <v>0.6120689655172413</v>
+        <v>0.6416666666666667</v>
       </c>
       <c r="F7" s="3">
-        <v>10.3</v>
+        <v>9.01</v>
       </c>
       <c r="G7" s="3">
-        <v>0.6976196057554538</v>
-      </c>
-      <c r="H7" s="3">
-        <v>4.984477107800576</v>
+        <v>5</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I7" s="3">
-        <v>5.302380394244546</v>
+        <v>0.6976196075069575</v>
       </c>
       <c r="J7" s="3">
-        <v>3.489500000000002</v>
+        <v>4.984477127902903</v>
       </c>
       <c r="K7" s="3">
-        <v>-5.14467691804052</v>
+        <v>5.302380392493043</v>
       </c>
       <c r="L7" s="3">
-        <v>7.166763644850975E-06</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
+        <v>1.164876168654569</v>
+      </c>
+      <c r="M7" s="3">
+        <v>0.3027107069978566</v>
+      </c>
+      <c r="N7" s="3">
+        <v>18.23776790244059</v>
+      </c>
+      <c r="O7" s="3">
+        <v>11.2410615417097</v>
+      </c>
+      <c r="P7" s="3">
+        <v>4.835123831345431</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>0.3027107069978566</v>
+      </c>
+      <c r="R7" s="3">
+        <v>3.728749283678181</v>
+      </c>
+      <c r="S7" s="3">
+        <v>57.30455632167204</v>
+      </c>
+      <c r="T7" s="3">
+        <v>4.241810845629632</v>
+      </c>
+      <c r="U7" s="3">
+        <v>5.42843681706123</v>
+      </c>
+      <c r="V7" s="3">
+        <v>0.3027107069978566</v>
+      </c>
+      <c r="W7" s="3">
+        <v>3.403400000000001</v>
+      </c>
+      <c r="X7" s="3">
+        <v>-5.568140156782245</v>
+      </c>
+      <c r="Y7" s="3">
+        <v>2.703085875570429E-06</v>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N7" s="3">
-        <v>62.84810638427734</v>
-      </c>
-      <c r="O7" s="3">
-        <v>55.03955078125</v>
-      </c>
-      <c r="P7" s="3">
-        <v>48.48752593994141</v>
-      </c>
-      <c r="Q7" s="3">
+      <c r="AA7" s="3">
+        <v>43.70171356201172</v>
+      </c>
+      <c r="AB7" s="3">
+        <v>27.25896072387695</v>
+      </c>
+      <c r="AC7" s="3">
+        <v>48.61517333984375</v>
+      </c>
+      <c r="AD7" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF7" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG7" s="3">
+        <v>0.05936180800199509</v>
+      </c>
+      <c r="AH7" s="3">
+        <v>0.2590552568435669</v>
+      </c>
+      <c r="AI7" s="3">
+        <v>0.8956759572029114</v>
+      </c>
+      <c r="AJ7" s="3">
+        <v>0.1856918781995773</v>
+      </c>
+      <c r="AK7" s="3">
+        <v>0.7018319964408875</v>
+      </c>
+      <c r="AL7" s="3">
+        <v>0.06777340173721313</v>
+      </c>
+      <c r="AM7" s="3">
+        <v>0.2325942814350128</v>
+      </c>
+      <c r="AN7" s="3">
+        <v>0.6252275705337524</v>
+      </c>
+      <c r="AO7" s="3">
+        <v>0.1200999021530151</v>
+      </c>
+      <c r="AP7" s="3">
+        <v>0.9302724003791809</v>
+      </c>
+      <c r="AQ7" s="3">
+        <v>0.9975115060806274</v>
+      </c>
+      <c r="AR7" s="3">
+        <v>0.8354297876358032</v>
+      </c>
+      <c r="AS7" s="3">
+        <v>0.8230787515640259</v>
+      </c>
+      <c r="AT7" s="3">
+        <v>0.7909397482872009</v>
+      </c>
+      <c r="AU7" s="3">
+        <v>-5.250341892242432</v>
+      </c>
+      <c r="AV7" s="3">
+        <v>96.24810791015625</v>
+      </c>
+      <c r="AW7" s="3">
+        <v>6.668382167816162</v>
+      </c>
+      <c r="AX7" s="3">
+        <v>480.6340000000002</v>
+      </c>
+      <c r="AY7" s="3">
+        <v>3.403400000000001</v>
+      </c>
+      <c r="AZ7" s="3">
+        <v>0.4839543874003267</v>
+      </c>
+      <c r="BA7" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB7" s="3">
+        <v>3.2734298364193</v>
+      </c>
+      <c r="BC7" s="3">
+        <v>0.7473966848422999</v>
+      </c>
+      <c r="BD7" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE7" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF7" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4cnn(C)c4)C3)C2)c1</t>
+          <t>CCCCCCC#Cc1cncc(N2CCC3(CN(C(=O)c4cc[nH]n4)C3)C2)c1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1109,44 +2093,169 @@
         <v>1</v>
       </c>
       <c r="E8" s="3">
-        <v>0.6403508771929824</v>
+        <v>0.6228070175438597</v>
       </c>
       <c r="F8" s="3">
-        <v>10.99</v>
+        <v>12.75</v>
       </c>
       <c r="G8" s="3">
-        <v>0.6976196057554538</v>
-      </c>
-      <c r="H8" s="3">
-        <v>4.984477107800576</v>
+        <v>5</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>KNN | KNN | DT | LGBM | ET</t>
+        </is>
       </c>
       <c r="I8" s="3">
-        <v>5.302380394244546</v>
+        <v>0.6976196075069575</v>
       </c>
       <c r="J8" s="3">
-        <v>3.489500000000002</v>
+        <v>4.984477127902903</v>
       </c>
       <c r="K8" s="3">
-        <v>-5.14467691804052</v>
+        <v>5.302380392493043</v>
       </c>
       <c r="L8" s="3">
-        <v>7.166763644850975E-06</v>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
+        <v>1.322618471770968</v>
+      </c>
+      <c r="M8" s="3">
+        <v>0.5542971669935401</v>
+      </c>
+      <c r="N8" s="3">
+        <v>52.04389975844849</v>
+      </c>
+      <c r="O8" s="3">
+        <v>74.57724903228805</v>
+      </c>
+      <c r="P8" s="3">
+        <v>4.677381528229032</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>0.5542971669935401</v>
+      </c>
+      <c r="R8" s="3">
+        <v>1.722645938188374</v>
+      </c>
+      <c r="S8" s="3">
+        <v>256.4725672714279</v>
+      </c>
+      <c r="T8" s="3">
+        <v>3.590959080921693</v>
+      </c>
+      <c r="U8" s="3">
+        <v>5.763803975536371</v>
+      </c>
+      <c r="V8" s="3">
+        <v>0.5542971669935401</v>
+      </c>
+      <c r="W8" s="3">
+        <v>3.479100000000002</v>
+      </c>
+      <c r="X8" s="3">
+        <v>-5.04957989485515</v>
+      </c>
+      <c r="Y8" s="3">
+        <v>8.921134870987701E-06</v>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
         <is>
           <t>Moderately Soluble</t>
         </is>
       </c>
-      <c r="N8" s="3">
-        <v>54.14443206787109</v>
-      </c>
-      <c r="O8" s="3">
-        <v>48.61449813842773</v>
-      </c>
-      <c r="P8" s="3">
-        <v>42.27074432373047</v>
-      </c>
-      <c r="Q8" s="3">
+      <c r="AA8" s="3">
+        <v>62.83623123168945</v>
+      </c>
+      <c r="AB8" s="3">
+        <v>60.1665153503418</v>
+      </c>
+      <c r="AC8" s="3">
+        <v>48.18215179443359</v>
+      </c>
+      <c r="AD8" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="3">
+        <v>2</v>
+      </c>
+      <c r="AF8" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG8" s="3">
+        <v>0.1282973736524582</v>
+      </c>
+      <c r="AH8" s="3">
+        <v>0.260791152715683</v>
+      </c>
+      <c r="AI8" s="3">
+        <v>0.8436020612716675</v>
+      </c>
+      <c r="AJ8" s="3">
+        <v>0.08913101255893707</v>
+      </c>
+      <c r="AK8" s="3">
+        <v>0.8110896944999695</v>
+      </c>
+      <c r="AL8" s="3">
+        <v>0.4075813293457031</v>
+      </c>
+      <c r="AM8" s="3">
+        <v>0.7175243496894836</v>
+      </c>
+      <c r="AN8" s="3">
+        <v>0.8229074478149414</v>
+      </c>
+      <c r="AO8" s="3">
+        <v>0.1541028469800949</v>
+      </c>
+      <c r="AP8" s="3">
+        <v>0.9670270085334778</v>
+      </c>
+      <c r="AQ8" s="3">
+        <v>0.999778151512146</v>
+      </c>
+      <c r="AR8" s="3">
+        <v>0.7362948656082153</v>
+      </c>
+      <c r="AS8" s="3">
+        <v>0.9462138414382935</v>
+      </c>
+      <c r="AT8" s="3">
+        <v>0.7763729095458984</v>
+      </c>
+      <c r="AU8" s="3">
+        <v>-4.844556331634521</v>
+      </c>
+      <c r="AV8" s="3">
+        <v>100.9472427368164</v>
+      </c>
+      <c r="AW8" s="3">
+        <v>9.599960327148438</v>
+      </c>
+      <c r="AX8" s="3">
+        <v>391.5190000000001</v>
+      </c>
+      <c r="AY8" s="3">
+        <v>3.479100000000002</v>
+      </c>
+      <c r="AZ8" s="3">
+        <v>0.6048053035660904</v>
+      </c>
+      <c r="BA8" s="3">
+        <v>4</v>
+      </c>
+      <c r="BB8" s="3">
+        <v>3.687574036396629</v>
+      </c>
+      <c r="BC8" s="3">
+        <v>0.7013806626225969</v>
+      </c>
+      <c r="BD8" s="3">
+        <v>2</v>
+      </c>
+      <c r="BE8" s="3">
+        <v>0</v>
+      </c>
+      <c r="BF8" s="3">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Filter dinitro compounds in nitro campaign outputs and add max-nitro scoring option
</commit_message>
<xml_diff>
--- a/outputs/generated/nitro_bioisostere_campaign/mol2mol_mmp/plain/mol2mol_mmp_plain_generated_optimal.xlsx
+++ b/outputs/generated/nitro_bioisostere_campaign/mol2mol_mmp/plain/mol2mol_mmp_plain_generated_optimal.xlsx
@@ -1069,7 +1069,7 @@
         <v>-4.697726188509208</v>
       </c>
       <c r="Y2" s="3">
-        <v>2.005736193847606E-05</v>
+        <v>2.005736193847605E-05</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1077,13 +1077,13 @@
         </is>
       </c>
       <c r="AA2" s="3">
-        <v>44.49736785888672</v>
+        <v>44.497368</v>
       </c>
       <c r="AB2" s="3">
-        <v>36.57278060913086</v>
+        <v>36.57278</v>
       </c>
       <c r="AC2" s="3">
-        <v>42.2242431640625</v>
+        <v>42.224243</v>
       </c>
       <c r="AD2" s="3">
         <v>0</v>
@@ -1095,55 +1095,55 @@
         <v>0</v>
       </c>
       <c r="AG2" s="3">
-        <v>0.1213474124670029</v>
+        <v>0.12134741</v>
       </c>
       <c r="AH2" s="3">
-        <v>0.3793679773807526</v>
+        <v>0.37936798</v>
       </c>
       <c r="AI2" s="3">
-        <v>0.6308319568634033</v>
+        <v>0.63083196</v>
       </c>
       <c r="AJ2" s="3">
-        <v>0.06799260526895523</v>
+        <v>0.067992605</v>
       </c>
       <c r="AK2" s="3">
-        <v>0.8862754702568054</v>
+        <v>0.8862755</v>
       </c>
       <c r="AL2" s="3">
-        <v>0.1875756233930588</v>
+        <v>0.18757562</v>
       </c>
       <c r="AM2" s="3">
-        <v>0.4857034087181091</v>
+        <v>0.4857034</v>
       </c>
       <c r="AN2" s="3">
-        <v>0.5998517274856567</v>
+        <v>0.5998517</v>
       </c>
       <c r="AO2" s="3">
-        <v>0.1621912717819214</v>
+        <v>0.16219127</v>
       </c>
       <c r="AP2" s="3">
-        <v>0.9689401388168335</v>
+        <v>0.9689401399999999</v>
       </c>
       <c r="AQ2" s="3">
-        <v>0.9997833967208862</v>
+        <v>0.9997834</v>
       </c>
       <c r="AR2" s="3">
-        <v>0.7327489852905273</v>
+        <v>0.732749</v>
       </c>
       <c r="AS2" s="3">
-        <v>0.9529389142990112</v>
+        <v>0.9529389</v>
       </c>
       <c r="AT2" s="3">
-        <v>0.8042116165161133</v>
+        <v>0.8042116</v>
       </c>
       <c r="AU2" s="3">
-        <v>-4.799037456512451</v>
+        <v>-4.7990375</v>
       </c>
       <c r="AV2" s="3">
-        <v>94.31733703613281</v>
+        <v>94.31734</v>
       </c>
       <c r="AW2" s="3">
-        <v>12.37920379638672</v>
+        <v>12.379204</v>
       </c>
       <c r="AX2" s="3">
         <v>382.5520000000002</v>
@@ -1258,13 +1258,13 @@
         </is>
       </c>
       <c r="AA3" s="3">
-        <v>56.6396598815918</v>
+        <v>56.63966</v>
       </c>
       <c r="AB3" s="3">
-        <v>48.72274017333984</v>
+        <v>48.72274</v>
       </c>
       <c r="AC3" s="3">
-        <v>43.81204986572266</v>
+        <v>43.81205</v>
       </c>
       <c r="AD3" s="3">
         <v>0</v>
@@ -1276,55 +1276,55 @@
         <v>0</v>
       </c>
       <c r="AG3" s="3">
-        <v>0.2192052155733109</v>
+        <v>0.21920522</v>
       </c>
       <c r="AH3" s="3">
-        <v>0.4016119837760925</v>
+        <v>0.40161198</v>
       </c>
       <c r="AI3" s="3">
-        <v>0.897729218006134</v>
+        <v>0.8977292</v>
       </c>
       <c r="AJ3" s="3">
-        <v>0.07054200768470764</v>
+        <v>0.07054201</v>
       </c>
       <c r="AK3" s="3">
-        <v>0.9418826103210449</v>
+        <v>0.9418826</v>
       </c>
       <c r="AL3" s="3">
-        <v>0.4947546124458313</v>
+        <v>0.4947546</v>
       </c>
       <c r="AM3" s="3">
-        <v>0.8435236811637878</v>
+        <v>0.8435237</v>
       </c>
       <c r="AN3" s="3">
-        <v>0.9229615330696106</v>
+        <v>0.92296153</v>
       </c>
       <c r="AO3" s="3">
-        <v>0.2877492904663086</v>
+        <v>0.2877493</v>
       </c>
       <c r="AP3" s="3">
-        <v>0.9939088821411133</v>
+        <v>0.9939089</v>
       </c>
       <c r="AQ3" s="3">
-        <v>0.9999846220016479</v>
+        <v>0.9999846</v>
       </c>
       <c r="AR3" s="3">
-        <v>0.726409375667572</v>
+        <v>0.7264094</v>
       </c>
       <c r="AS3" s="3">
-        <v>0.9672144651412964</v>
+        <v>0.96721447</v>
       </c>
       <c r="AT3" s="3">
-        <v>0.9312014579772949</v>
+        <v>0.93120146</v>
       </c>
       <c r="AU3" s="3">
-        <v>-4.826889991760254</v>
+        <v>-4.82689</v>
       </c>
       <c r="AV3" s="3">
-        <v>102.379753112793</v>
+        <v>102.37975</v>
       </c>
       <c r="AW3" s="3">
-        <v>6.813174247741699</v>
+        <v>6.8131742</v>
       </c>
       <c r="AX3" s="3">
         <v>461.5660000000003</v>
@@ -1395,7 +1395,7 @@
         <v>0.8836030068125652</v>
       </c>
       <c r="M4" s="3">
-        <v>0.1803645338738968</v>
+        <v>0.1803645338738967</v>
       </c>
       <c r="N4" s="3">
         <v>8.32240433842561</v>
@@ -1407,7 +1407,7 @@
         <v>5.116396993187434</v>
       </c>
       <c r="Q4" s="3">
-        <v>0.1803645338738968</v>
+        <v>0.1803645338738967</v>
       </c>
       <c r="R4" s="3">
         <v>3.38913228359138</v>
@@ -1422,7 +1422,7 @@
         <v>5.469911479580272</v>
       </c>
       <c r="V4" s="3">
-        <v>0.1803645338738968</v>
+        <v>0.1803645338738967</v>
       </c>
       <c r="W4" s="3">
         <v>3.478700000000003</v>
@@ -1439,13 +1439,13 @@
         </is>
       </c>
       <c r="AA4" s="3">
-        <v>53.13448333740234</v>
+        <v>53.134483</v>
       </c>
       <c r="AB4" s="3">
-        <v>56.53021240234375</v>
+        <v>56.530212</v>
       </c>
       <c r="AC4" s="3">
-        <v>44.11494064331055</v>
+        <v>44.11494</v>
       </c>
       <c r="AD4" s="3">
         <v>0</v>
@@ -1457,55 +1457,55 @@
         <v>0</v>
       </c>
       <c r="AG4" s="3">
-        <v>0.2469469308853149</v>
+        <v>0.24694693</v>
       </c>
       <c r="AH4" s="3">
-        <v>0.2810777425765991</v>
+        <v>0.28107774</v>
       </c>
       <c r="AI4" s="3">
-        <v>0.6463785171508789</v>
+        <v>0.6463785</v>
       </c>
       <c r="AJ4" s="3">
-        <v>0.05409278720617294</v>
+        <v>0.054092787</v>
       </c>
       <c r="AK4" s="3">
-        <v>0.8009153604507446</v>
+        <v>0.80091536</v>
       </c>
       <c r="AL4" s="3">
-        <v>0.206072524189949</v>
+        <v>0.20607252</v>
       </c>
       <c r="AM4" s="3">
-        <v>0.5045340061187744</v>
+        <v>0.504534</v>
       </c>
       <c r="AN4" s="3">
-        <v>0.5027914643287659</v>
+        <v>0.50279146</v>
       </c>
       <c r="AO4" s="3">
-        <v>0.09001477062702179</v>
+        <v>0.09001476999999999</v>
       </c>
       <c r="AP4" s="3">
-        <v>0.9486678838729858</v>
+        <v>0.9486679</v>
       </c>
       <c r="AQ4" s="3">
-        <v>0.9999431371688843</v>
+        <v>0.99994314</v>
       </c>
       <c r="AR4" s="3">
-        <v>0.7472778558731079</v>
+        <v>0.74727786</v>
       </c>
       <c r="AS4" s="3">
-        <v>0.9748571515083313</v>
+        <v>0.97485715</v>
       </c>
       <c r="AT4" s="3">
-        <v>0.7642152309417725</v>
+        <v>0.76421523</v>
       </c>
       <c r="AU4" s="3">
-        <v>-4.632003784179688</v>
+        <v>-4.632004</v>
       </c>
       <c r="AV4" s="3">
-        <v>97.15895843505859</v>
+        <v>97.15895999999999</v>
       </c>
       <c r="AW4" s="3">
-        <v>10.61889266967773</v>
+        <v>10.618893</v>
       </c>
       <c r="AX4" s="3">
         <v>395.5470000000003</v>
@@ -1582,7 +1582,7 @@
         <v>14.99202021366446</v>
       </c>
       <c r="O5" s="3">
-        <v>9.017290093260467</v>
+        <v>9.017290093260469</v>
       </c>
       <c r="P5" s="3">
         <v>4.912103278568816</v>
@@ -1612,7 +1612,7 @@
         <v>-5.14467691804052</v>
       </c>
       <c r="Y5" s="3">
-        <v>7.166763644850975E-06</v>
+        <v>7.166763644850976E-06</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1620,13 +1620,13 @@
         </is>
       </c>
       <c r="AA5" s="3">
-        <v>54.14443206787109</v>
+        <v>54.144432</v>
       </c>
       <c r="AB5" s="3">
-        <v>48.61449813842773</v>
+        <v>48.6145</v>
       </c>
       <c r="AC5" s="3">
-        <v>42.2707405090332</v>
+        <v>42.27074</v>
       </c>
       <c r="AD5" s="3">
         <v>0</v>
@@ -1638,55 +1638,55 @@
         <v>0</v>
       </c>
       <c r="AG5" s="3">
-        <v>0.1222689300775528</v>
+        <v>0.12226893</v>
       </c>
       <c r="AH5" s="3">
-        <v>0.2155998200178146</v>
+        <v>0.21559982</v>
       </c>
       <c r="AI5" s="3">
-        <v>0.8456916809082031</v>
+        <v>0.8456917</v>
       </c>
       <c r="AJ5" s="3">
-        <v>0.06358656287193298</v>
+        <v>0.06358656</v>
       </c>
       <c r="AK5" s="3">
-        <v>0.760409951210022</v>
+        <v>0.76040995</v>
       </c>
       <c r="AL5" s="3">
-        <v>0.2809678912162781</v>
+        <v>0.2809679</v>
       </c>
       <c r="AM5" s="3">
-        <v>0.5562871098518372</v>
+        <v>0.5562871</v>
       </c>
       <c r="AN5" s="3">
-        <v>0.7078112363815308</v>
+        <v>0.70781124</v>
       </c>
       <c r="AO5" s="3">
-        <v>0.05011356994509697</v>
+        <v>0.05011357</v>
       </c>
       <c r="AP5" s="3">
-        <v>0.9613454937934875</v>
+        <v>0.9613455</v>
       </c>
       <c r="AQ5" s="3">
-        <v>0.9999285936355591</v>
+        <v>0.9999285999999999</v>
       </c>
       <c r="AR5" s="3">
-        <v>0.8209438323974609</v>
+        <v>0.82094383</v>
       </c>
       <c r="AS5" s="3">
-        <v>0.968595027923584</v>
+        <v>0.968595</v>
       </c>
       <c r="AT5" s="3">
-        <v>0.7425563931465149</v>
+        <v>0.7425564</v>
       </c>
       <c r="AU5" s="3">
-        <v>-4.84219217300415</v>
+        <v>-4.842192</v>
       </c>
       <c r="AV5" s="3">
-        <v>98.20294189453125</v>
+        <v>98.20294</v>
       </c>
       <c r="AW5" s="3">
-        <v>9.877103805541992</v>
+        <v>9.877103999999999</v>
       </c>
       <c r="AX5" s="3">
         <v>405.5460000000002</v>
@@ -1793,7 +1793,7 @@
         <v>-5.14467691804052</v>
       </c>
       <c r="Y6" s="3">
-        <v>7.166763644850975E-06</v>
+        <v>7.166763644850976E-06</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -1801,13 +1801,13 @@
         </is>
       </c>
       <c r="AA6" s="3">
-        <v>62.84810638427734</v>
+        <v>62.848106</v>
       </c>
       <c r="AB6" s="3">
-        <v>55.03955078125</v>
+        <v>55.03955</v>
       </c>
       <c r="AC6" s="3">
-        <v>48.48752593994141</v>
+        <v>48.487526</v>
       </c>
       <c r="AD6" s="3">
         <v>0</v>
@@ -1819,55 +1819,55 @@
         <v>0</v>
       </c>
       <c r="AG6" s="3">
-        <v>0.1596864759922028</v>
+        <v>0.15968648</v>
       </c>
       <c r="AH6" s="3">
-        <v>0.2792690992355347</v>
+        <v>0.2792691</v>
       </c>
       <c r="AI6" s="3">
-        <v>0.8238638043403625</v>
+        <v>0.8238638</v>
       </c>
       <c r="AJ6" s="3">
-        <v>0.0565599612891674</v>
+        <v>0.05655996</v>
       </c>
       <c r="AK6" s="3">
-        <v>0.8657090067863464</v>
+        <v>0.865709</v>
       </c>
       <c r="AL6" s="3">
-        <v>0.4318308234214783</v>
+        <v>0.43183082</v>
       </c>
       <c r="AM6" s="3">
-        <v>0.7112659215927124</v>
+        <v>0.7112659</v>
       </c>
       <c r="AN6" s="3">
-        <v>0.8083459734916687</v>
+        <v>0.808346</v>
       </c>
       <c r="AO6" s="3">
-        <v>0.1134422272443771</v>
+        <v>0.11344223</v>
       </c>
       <c r="AP6" s="3">
-        <v>0.987573504447937</v>
+        <v>0.9875735</v>
       </c>
       <c r="AQ6" s="3">
-        <v>0.9999877214431763</v>
+        <v>0.9999877</v>
       </c>
       <c r="AR6" s="3">
-        <v>0.7667804956436157</v>
+        <v>0.7667805</v>
       </c>
       <c r="AS6" s="3">
-        <v>0.9786069989204407</v>
+        <v>0.978607</v>
       </c>
       <c r="AT6" s="3">
-        <v>0.8238350749015808</v>
+        <v>0.8238351</v>
       </c>
       <c r="AU6" s="3">
-        <v>-4.787118434906006</v>
+        <v>-4.7871184</v>
       </c>
       <c r="AV6" s="3">
-        <v>99.26639556884766</v>
+        <v>99.266396</v>
       </c>
       <c r="AW6" s="3">
-        <v>10.56526756286621</v>
+        <v>10.565268</v>
       </c>
       <c r="AX6" s="3">
         <v>405.5460000000002</v>
@@ -1938,7 +1938,7 @@
         <v>1.164876168654569</v>
       </c>
       <c r="M7" s="3">
-        <v>0.3027107069978566</v>
+        <v>0.3027107069978565</v>
       </c>
       <c r="N7" s="3">
         <v>18.23776790244059</v>
@@ -1950,7 +1950,7 @@
         <v>4.835123831345431</v>
       </c>
       <c r="Q7" s="3">
-        <v>0.3027107069978566</v>
+        <v>0.3027107069978565</v>
       </c>
       <c r="R7" s="3">
         <v>3.728749283678181</v>
@@ -1965,7 +1965,7 @@
         <v>5.42843681706123</v>
       </c>
       <c r="V7" s="3">
-        <v>0.3027107069978566</v>
+        <v>0.3027107069978565</v>
       </c>
       <c r="W7" s="3">
         <v>3.403400000000001</v>
@@ -1982,13 +1982,13 @@
         </is>
       </c>
       <c r="AA7" s="3">
-        <v>43.70171356201172</v>
+        <v>43.701714</v>
       </c>
       <c r="AB7" s="3">
-        <v>27.25896072387695</v>
+        <v>27.25896</v>
       </c>
       <c r="AC7" s="3">
-        <v>48.61517333984375</v>
+        <v>48.615173</v>
       </c>
       <c r="AD7" s="3">
         <v>0</v>
@@ -2000,55 +2000,55 @@
         <v>0</v>
       </c>
       <c r="AG7" s="3">
-        <v>0.05936180800199509</v>
+        <v>0.059361808</v>
       </c>
       <c r="AH7" s="3">
-        <v>0.2590552568435669</v>
+        <v>0.25905526</v>
       </c>
       <c r="AI7" s="3">
-        <v>0.8956759572029114</v>
+        <v>0.89567596</v>
       </c>
       <c r="AJ7" s="3">
-        <v>0.1856918781995773</v>
+        <v>0.18569188</v>
       </c>
       <c r="AK7" s="3">
-        <v>0.7018319964408875</v>
+        <v>0.701832</v>
       </c>
       <c r="AL7" s="3">
-        <v>0.06777340173721313</v>
+        <v>0.0677734</v>
       </c>
       <c r="AM7" s="3">
-        <v>0.2325942814350128</v>
+        <v>0.23259428</v>
       </c>
       <c r="AN7" s="3">
-        <v>0.6252275705337524</v>
+        <v>0.6252276</v>
       </c>
       <c r="AO7" s="3">
-        <v>0.1200999021530151</v>
+        <v>0.1200999</v>
       </c>
       <c r="AP7" s="3">
-        <v>0.9302724003791809</v>
+        <v>0.9302724</v>
       </c>
       <c r="AQ7" s="3">
-        <v>0.9975115060806274</v>
+        <v>0.9975115</v>
       </c>
       <c r="AR7" s="3">
-        <v>0.8354297876358032</v>
+        <v>0.8354298</v>
       </c>
       <c r="AS7" s="3">
-        <v>0.8230787515640259</v>
+        <v>0.82307875</v>
       </c>
       <c r="AT7" s="3">
-        <v>0.7909397482872009</v>
+        <v>0.7909397500000001</v>
       </c>
       <c r="AU7" s="3">
-        <v>-5.250341892242432</v>
+        <v>-5.250342</v>
       </c>
       <c r="AV7" s="3">
-        <v>96.24810791015625</v>
+        <v>96.24811</v>
       </c>
       <c r="AW7" s="3">
-        <v>6.668382167816162</v>
+        <v>6.668382</v>
       </c>
       <c r="AX7" s="3">
         <v>480.6340000000002</v>
@@ -2163,13 +2163,13 @@
         </is>
       </c>
       <c r="AA8" s="3">
-        <v>62.83623123168945</v>
+        <v>62.83623</v>
       </c>
       <c r="AB8" s="3">
-        <v>60.1665153503418</v>
+        <v>60.166515</v>
       </c>
       <c r="AC8" s="3">
-        <v>48.18215179443359</v>
+        <v>48.18215</v>
       </c>
       <c r="AD8" s="3">
         <v>0</v>
@@ -2181,55 +2181,55 @@
         <v>0</v>
       </c>
       <c r="AG8" s="3">
-        <v>0.1282973736524582</v>
+        <v>0.12829737</v>
       </c>
       <c r="AH8" s="3">
-        <v>0.260791152715683</v>
+        <v>0.26079115</v>
       </c>
       <c r="AI8" s="3">
-        <v>0.8436020612716675</v>
+        <v>0.84360206</v>
       </c>
       <c r="AJ8" s="3">
-        <v>0.08913101255893707</v>
+        <v>0.08913101</v>
       </c>
       <c r="AK8" s="3">
-        <v>0.8110896944999695</v>
+        <v>0.8110897</v>
       </c>
       <c r="AL8" s="3">
-        <v>0.4075813293457031</v>
+        <v>0.40758133</v>
       </c>
       <c r="AM8" s="3">
-        <v>0.7175243496894836</v>
+        <v>0.71752435</v>
       </c>
       <c r="AN8" s="3">
-        <v>0.8229074478149414</v>
+        <v>0.82290745</v>
       </c>
       <c r="AO8" s="3">
-        <v>0.1541028469800949</v>
+        <v>0.15410285</v>
       </c>
       <c r="AP8" s="3">
-        <v>0.9670270085334778</v>
+        <v>0.967027</v>
       </c>
       <c r="AQ8" s="3">
-        <v>0.999778151512146</v>
+        <v>0.99977815</v>
       </c>
       <c r="AR8" s="3">
-        <v>0.7362948656082153</v>
+        <v>0.73629487</v>
       </c>
       <c r="AS8" s="3">
-        <v>0.9462138414382935</v>
+        <v>0.94621384</v>
       </c>
       <c r="AT8" s="3">
-        <v>0.7763729095458984</v>
+        <v>0.7763729</v>
       </c>
       <c r="AU8" s="3">
-        <v>-4.844556331634521</v>
+        <v>-4.8445563</v>
       </c>
       <c r="AV8" s="3">
-        <v>100.9472427368164</v>
+        <v>100.94724</v>
       </c>
       <c r="AW8" s="3">
-        <v>9.599960327148438</v>
+        <v>9.599959999999999</v>
       </c>
       <c r="AX8" s="3">
         <v>391.5190000000001</v>

</xml_diff>